<commit_message>
docs: populate severity and impact fields for DEF-018
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.4.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.4.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="B1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -1923,9 +1923,21 @@
           <t>npm test (full suite)</t>
         </is>
       </c>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="6" t="n"/>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>None (Test environment transient failure)</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1946,8 +1958,16 @@
           <t>Pending. Recorded in docs/evidence/M3-indexes/INDEX_provisioning_script_NV.txt (PR #98).</t>
         </is>
       </c>
-      <c r="N28" s="6" t="n"/>
-      <c r="O28" s="6" t="n"/>
+      <c r="N28" s="6" t="inlineStr">
+        <is>
+          <t>Transient CI instability</t>
+        </is>
+      </c>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>Ethan Lindsay</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="B10:O28"/>

</xml_diff>

<commit_message>
docs: DEF-018 review fixes: finder, facts, relation, impact, fix plan, owner; B2 note
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.4.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.4.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register. | Version 0.4 (14/10/2026). Adds DEF-018 (an intermittent npm test failure in the PR #98 build: 3 failures, test names not captured). DEF-001 to DEF-017 unchanged. | Version 0.3 (12/10/2026). Adds DEF-017 (the unique index on users.email is absent on the test cluster; FR-1.1 relies on it alone), raised by E. Lindsay; DEF-014 and DEF-015 cell E updated with the observed index absence from the test-cluster listing. DEF-001 to DEF-016 otherwise unchanged. Version 0.2 (12/10/2026). Adds DEF-005 to DEF-016: DEF-007 to DEF-010, DEF-014, and DEF-015 from M3 integration testing (R. van der Merwe); DEF-005, DEF-006, DEF-011 to DEF-013, and DEF-016 raised by E. Lindsay. DEF-001 to DEF-004 unchanged. Version 0.1 (11/10/2026). Register created with DEF-001 to DEF-004.</t>
+          <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register. | Version 0.4 (14/10/2026). Adds DEF-018 (an unexplained npm test failure in the PR #98 build: 3 failures, test names not captured), raised by R. van der Merwe. DEF-001 to DEF-017 unchanged. Version 0.3 (12/10/2026). Adds DEF-017 (the unique index on users.email is absent on the test cluster; FR-1.1 relies on it alone), raised by E. Lindsay; DEF-014 and DEF-015 cell E updated with the observed index absence from the test-cluster listing. DEF-001 to DEF-016 otherwise unchanged. Version 0.2 (12/10/2026). Adds DEF-005 to DEF-016: DEF-007 to DEF-010, DEF-014, and DEF-015 from M3 integration testing (R. van der Merwe); DEF-005, DEF-006, DEF-011 to DEF-013, and DEF-016 raised by E. Lindsay. DEF-001 to DEF-004 unchanged. Version 0.1 (11/10/2026). Register created with DEF-001 to DEF-004.</t>
         </is>
       </c>
     </row>
@@ -1910,17 +1910,17 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Full-suite run during the PR #98 build (the first full run after tests/indexProvisioning.test.js was added)</t>
+          <t>Ethan, during the PR #98 build on 13/10/2026 (UTC)</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>npm test failed intermittently: the first full run after the new test file was added gave 194 tests, 183 pass, 3 fail, 8 skipped. The failing test names were not captured. The 15 later full-suite runs all passed. It was not re-run to green. Cause unknown.</t>
+          <t>The first full npm test run after tests/indexProvisioning.test.js was added gave 194 tests, 183 pass, 3 fail, 8 skipped. The failing test names were not captured. Not known whether the three failures were in #98's new tests or the existing suite. 15 later runs each gave 194 tests, 186 pass, 8 skipped, 0 fail. It was not re-run to green. One unexplained failure, not reproduced. Cause unknown. Recorded in docs/evidence/M3-indexes/INDEX_provisioning_script_NV.txt (PR #98).</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>npm test (full suite)</t>
+          <t>npm test (full suite). Not known whether related to DEF-013 or DEF-016: the failing tests were not captured.</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>None (Test environment transient failure)</t>
+          <t>npm test is the CI gate; an unexplained failure can't be told apart from a real fault and invites re-running until green; if the failures included DEF-013's session-cookie test, the uncertainty is about a security control.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Capture test names and messages with a reporter, decide whether the cause is in the test setup or the app if it recurs, fix it without weakening any assertion, and never re-run until green.</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr">
@@ -1955,17 +1955,17 @@
       </c>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>Pending. Recorded in docs/evidence/M3-indexes/INDEX_provisioning_script_NV.txt (PR #98).</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>Transient CI instability</t>
+          <t>Not release-blocking (S3). Residual: the cause of three test failures is unknown, and they cannot be ruled out as a real fault.</t>
         </is>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
-          <t>Ethan Lindsay</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>

</xml_diff>